<commit_message>
Actualitzat a PiG4 GestioProductes i PerduesGuanysTab.
--HG--
branch : Proves PiG
</commit_message>
<xml_diff>
--- a/Docs/Moviments-Fons Amb Cartera.xlsx
+++ b/Docs/Moviments-Fons Amb Cartera.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\_Actiu\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0645D639-FB52-4928-A666-49935700CCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0749296F-A9C9-4299-A0C1-3C039B96B465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="689" firstSheet="1" activeTab="1" xr2:uid="{67C9267C-8DE9-4BF2-8230-BF48900302D9}"/>
+    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12576" tabRatio="689" xr2:uid="{67C9267C-8DE9-4BF2-8230-BF48900302D9}"/>
   </bookViews>
   <sheets>
     <sheet name="28-Euro Fund" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="67">
   <si>
     <t>Traspàs C</t>
   </si>
@@ -167,21 +167,6 @@
     <t>V</t>
   </si>
   <si>
-    <t>Prod</t>
-  </si>
-  <si>
-    <t>Venudes en</t>
-  </si>
-  <si>
-    <t>Id: 1229</t>
-  </si>
-  <si>
-    <t>Id: 1278</t>
-  </si>
-  <si>
-    <t>bbva</t>
-  </si>
-  <si>
     <t>Brut</t>
   </si>
   <si>
@@ -251,24 +236,6 @@
     <t>Import comp cartera</t>
   </si>
   <si>
-    <t>1042-DWS Floating Rate Notes LC</t>
-  </si>
-  <si>
-    <t>1043-Global Technology A-Acc-USD H</t>
-  </si>
-  <si>
-    <t>Arcelor</t>
-  </si>
-  <si>
-    <t>Amb Desp</t>
-  </si>
-  <si>
-    <t>Arcelor Trade</t>
-  </si>
-  <si>
-    <t>Desp</t>
-  </si>
-  <si>
     <t>PiG 1251</t>
   </si>
   <si>
@@ -285,6 +252,12 @@
   </si>
   <si>
     <t>DWS Floating Rate Notes LC</t>
+  </si>
+  <si>
+    <t>Compra 1273</t>
+  </si>
+  <si>
+    <t>compra 1275</t>
   </si>
 </sst>
 </file>
@@ -611,17 +584,11 @@
     <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -675,17 +642,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="166" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="170" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="165" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1003,7 +970,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.90625" bestFit="1" customWidth="1"/>
@@ -1038,7 +1005,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="L1" s="46" t="s">
         <v>11</v>
@@ -1054,7 +1021,7 @@
       <c r="C2" s="3">
         <v>44473</v>
       </c>
-      <c r="D2" s="71">
+      <c r="D2" s="70">
         <v>24.54</v>
       </c>
       <c r="E2" s="48">
@@ -1082,7 +1049,7 @@
       </c>
       <c r="L2" s="4">
         <f t="shared" ref="L2:L8" si="0">(E$10-E2)*I2</f>
-        <v>149.72603039999993</v>
+        <v>150.00410879999993</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -1095,7 +1062,7 @@
       <c r="C3" s="3">
         <v>44496</v>
       </c>
-      <c r="D3" s="71">
+      <c r="D3" s="70">
         <v>34.723999999999997</v>
       </c>
       <c r="E3" s="48">
@@ -1119,7 +1086,7 @@
       </c>
       <c r="L3" s="4">
         <f t="shared" si="0"/>
-        <v>885.98980479999966</v>
+        <v>887.62530519999973</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -1132,7 +1099,7 @@
       <c r="C4" s="3">
         <v>44524</v>
       </c>
-      <c r="D4" s="71">
+      <c r="D4" s="70">
         <v>46.265999999999998</v>
       </c>
       <c r="E4" s="48">
@@ -1156,7 +1123,7 @@
       </c>
       <c r="L4" s="4">
         <f t="shared" si="0"/>
-        <v>1189.2351437999994</v>
+        <v>1191.4142723999994</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -1169,7 +1136,7 @@
       <c r="C5" s="3">
         <v>44725</v>
       </c>
-      <c r="D5" s="71">
+      <c r="D5" s="70">
         <v>23.23</v>
       </c>
       <c r="E5" s="48">
@@ -1193,7 +1160,7 @@
       </c>
       <c r="L5" s="4">
         <f t="shared" si="0"/>
-        <v>631.36584700000003</v>
+        <v>632.45997999999997</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -1206,7 +1173,7 @@
       <c r="C6" s="3">
         <v>44893</v>
       </c>
-      <c r="D6" s="71">
+      <c r="D6" s="70">
         <v>21.81</v>
       </c>
       <c r="E6" s="48">
@@ -1230,7 +1197,7 @@
       </c>
       <c r="L6" s="4">
         <f t="shared" si="0"/>
-        <v>587.60720099999958</v>
+        <v>588.63445199999956</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -1243,7 +1210,7 @@
       <c r="C7" s="3">
         <v>44893</v>
       </c>
-      <c r="D7" s="71">
+      <c r="D7" s="70">
         <v>18.635999999999999</v>
       </c>
       <c r="E7" s="48">
@@ -1267,7 +1234,7 @@
       </c>
       <c r="L7" s="4">
         <f t="shared" si="0"/>
-        <v>501.68298359999983</v>
+        <v>502.56073919999983</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -1280,7 +1247,7 @@
       <c r="C8" s="3">
         <v>44939</v>
       </c>
-      <c r="D8" s="71">
+      <c r="D8" s="70">
         <v>5.8719999999999999</v>
       </c>
       <c r="E8" s="48">
@@ -1304,7 +1271,7 @@
       </c>
       <c r="L8" s="4">
         <f t="shared" si="0"/>
-        <v>152.73717919999999</v>
+        <v>153.01375039999999</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -1317,7 +1284,7 @@
       <c r="C9" s="3">
         <v>45495</v>
       </c>
-      <c r="D9" s="71">
+      <c r="D9" s="70">
         <v>18.635999999999999</v>
       </c>
       <c r="E9" s="48">
@@ -1334,7 +1301,7 @@
       <c r="I9" s="4"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B10" s="72" t="s">
+      <c r="B10" s="71" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="45"/>
@@ -1343,13 +1310,13 @@
         <v>156.44199999999998</v>
       </c>
       <c r="E10" s="69">
-        <v>460.46199999999999</v>
+        <v>460.50909999999999</v>
       </c>
       <c r="F10" s="45"/>
       <c r="G10" s="45"/>
       <c r="H10" s="9">
         <f>D10*E10</f>
-        <v>72035.596203999987</v>
+        <v>72042.964622199986</v>
       </c>
       <c r="I10" s="4"/>
     </row>
@@ -1365,22 +1332,17 @@
       </c>
       <c r="L11" s="4">
         <f>SUM(L2:L9)</f>
-        <v>4098.3441897999992</v>
+        <v>4105.712607999998</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="J12" s="8"/>
       <c r="K12" s="8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="L12" s="69">
         <f>+J11+L11</f>
-        <v>4520.2669569999989</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="L14">
-        <v>4075.19</v>
+        <v>4527.6353751999977</v>
       </c>
     </row>
   </sheetData>
@@ -1413,10 +1375,10 @@
     <col min="15" max="15" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.6328125" customWidth="1"/>
-    <col min="18" max="18" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.26953125" customWidth="1"/>
     <col min="19" max="19" width="13.90625" customWidth="1"/>
     <col min="20" max="20" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="29" customHeight="1" x14ac:dyDescent="0.35">
@@ -1447,11 +1409,11 @@
       <c r="I1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="98" t="s">
+      <c r="J1" s="96" t="s">
         <v>13</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>8</v>
@@ -1475,13 +1437,13 @@
         <v>19</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="U1" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
@@ -1512,7 +1474,7 @@
       <c r="I2" s="42">
         <v>18.6356</v>
       </c>
-      <c r="J2" s="99">
+      <c r="J2" s="97">
         <v>321.66890000000001</v>
       </c>
       <c r="K2" s="20">
@@ -1579,7 +1541,7 @@
       <c r="I3" s="43">
         <v>18.635999999999999</v>
       </c>
-      <c r="J3" s="94"/>
+      <c r="J3" s="92"/>
       <c r="K3" s="24"/>
       <c r="L3" s="43">
         <f>I2</f>
@@ -1628,7 +1590,7 @@
       <c r="I4" s="42">
         <v>23.23</v>
       </c>
-      <c r="J4" s="99">
+      <c r="J4" s="97">
         <v>152.5463</v>
       </c>
       <c r="K4" s="20">
@@ -1664,7 +1626,7 @@
       </c>
       <c r="S4" s="21">
         <f>N4*G$16-Q4</f>
-        <v>7910.9006011730071</v>
+        <v>7911.9947153330086</v>
       </c>
       <c r="T4" s="21">
         <f>T5/I5*L4</f>
@@ -1672,7 +1634,7 @@
       </c>
       <c r="U4" s="21">
         <f>R4+S4</f>
-        <v>7911.0357342517018</v>
+        <v>7912.1298484117033</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
@@ -1695,7 +1657,7 @@
       <c r="I5" s="43">
         <v>18.635999999999999</v>
       </c>
-      <c r="J5" s="94"/>
+      <c r="J5" s="92"/>
       <c r="K5" s="24"/>
       <c r="L5" s="43">
         <f>I5-L3</f>
@@ -1744,7 +1706,7 @@
       <c r="I6" s="42">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="J6" s="99">
+      <c r="J6" s="97">
         <v>2.8999999999999998E-3</v>
       </c>
       <c r="K6" s="20">
@@ -1780,7 +1742,7 @@
       </c>
       <c r="S6" s="21">
         <f>N6*G$16-Q6</f>
-        <v>0.13123080000402462</v>
+        <v>0.13124964000402461</v>
       </c>
       <c r="T6" s="21">
         <f>T7/I7*L6</f>
@@ -1788,7 +1750,7 @@
       </c>
       <c r="U6" s="21">
         <f>R6+S6</f>
-        <v>0.13123080000402462</v>
+        <v>0.13124964000402461</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
@@ -1819,7 +1781,7 @@
       <c r="I7" s="42">
         <v>2.0112999999999999</v>
       </c>
-      <c r="J7" s="99">
+      <c r="J7" s="97">
         <v>14.956799999999999</v>
       </c>
       <c r="K7" s="20">
@@ -1855,7 +1817,7 @@
       </c>
       <c r="S7" s="21">
         <f t="shared" ref="S7:S15" si="7">N7*G$16-Q7</f>
-        <v>653.01605262075691</v>
+        <v>653.110784850757</v>
       </c>
       <c r="T7" s="21">
         <f t="shared" ref="T7:T15" si="8">T8/I8*L7</f>
@@ -1863,7 +1825,7 @@
       </c>
       <c r="U7" s="21">
         <f t="shared" ref="U7:U15" si="9">R7+S7</f>
-        <v>653.01605262075691</v>
+        <v>653.110784850757</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
@@ -1894,7 +1856,7 @@
       <c r="I8" s="42">
         <v>21.81</v>
       </c>
-      <c r="J8" s="99">
+      <c r="J8" s="97">
         <v>158.67240000000001</v>
       </c>
       <c r="K8" s="20">
@@ -1930,7 +1892,7 @@
       </c>
       <c r="S8" s="21">
         <f t="shared" si="7"/>
-        <v>7145.3181962202043</v>
+        <v>7146.3454472202038</v>
       </c>
       <c r="T8" s="21">
         <f t="shared" si="8"/>
@@ -1938,7 +1900,7 @@
       </c>
       <c r="U8" s="21">
         <f t="shared" si="9"/>
-        <v>7145.3181962202043</v>
+        <v>7146.3454472202038</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.35">
@@ -1969,7 +1931,7 @@
       <c r="I9" s="42">
         <v>24.54</v>
       </c>
-      <c r="J9" s="99">
+      <c r="J9" s="97">
         <v>226.48509999999999</v>
       </c>
       <c r="K9" s="20">
@@ -2005,7 +1967,7 @@
       </c>
       <c r="S9" s="21">
         <f t="shared" si="7"/>
-        <v>6817.5977297409991</v>
+        <v>6818.7535637409983</v>
       </c>
       <c r="T9" s="21">
         <f t="shared" si="8"/>
@@ -2013,7 +1975,7 @@
       </c>
       <c r="U9" s="21">
         <f t="shared" si="9"/>
-        <v>6817.5977297409991</v>
+        <v>6818.7535637409983</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.35">
@@ -2044,7 +2006,7 @@
       <c r="I10" s="42">
         <v>1.1525000000000001</v>
       </c>
-      <c r="J10" s="99">
+      <c r="J10" s="97">
         <v>18.2224</v>
       </c>
       <c r="K10" s="20">
@@ -2080,7 +2042,7 @@
       </c>
       <c r="S10" s="21">
         <f t="shared" si="7"/>
-        <v>170.06118947251224</v>
+        <v>170.11547222251221</v>
       </c>
       <c r="T10" s="21">
         <f t="shared" si="8"/>
@@ -2088,7 +2050,7 @@
       </c>
       <c r="U10" s="21">
         <f t="shared" si="9"/>
-        <v>170.06118947251224</v>
+        <v>170.11547222251221</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.35">
@@ -2119,7 +2081,7 @@
       <c r="I11" s="42">
         <v>46.265999999999998</v>
       </c>
-      <c r="J11" s="99">
+      <c r="J11" s="97">
         <v>396.34890000000001</v>
       </c>
       <c r="K11" s="20">
@@ -2155,7 +2117,7 @@
       </c>
       <c r="S11" s="21">
         <f t="shared" si="7"/>
-        <v>13459.990823796707</v>
+        <v>13462.169952396704</v>
       </c>
       <c r="T11" s="21">
         <f t="shared" si="8"/>
@@ -2163,7 +2125,7 @@
       </c>
       <c r="U11" s="21">
         <f t="shared" si="9"/>
-        <v>13459.990823796707</v>
+        <v>13462.169952396704</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.35">
@@ -2194,7 +2156,7 @@
       <c r="I12" s="42">
         <v>29.760999999999999</v>
       </c>
-      <c r="J12" s="99">
+      <c r="J12" s="97">
         <v>22.006</v>
       </c>
       <c r="K12" s="20">
@@ -2230,7 +2192,7 @@
       </c>
       <c r="S12" s="21">
         <f t="shared" si="7"/>
-        <v>8192.5999779820704</v>
+        <v>8194.0017210820697</v>
       </c>
       <c r="T12" s="21">
         <f t="shared" si="8"/>
@@ -2238,7 +2200,7 @@
       </c>
       <c r="U12" s="21">
         <f t="shared" si="9"/>
-        <v>8192.5999779820704</v>
+        <v>8194.0017210820697</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.35">
@@ -2269,7 +2231,7 @@
       <c r="I13" s="42">
         <v>0.64380000000000004</v>
       </c>
-      <c r="J13" s="99">
+      <c r="J13" s="97">
         <v>13.0237</v>
       </c>
       <c r="K13" s="20">
@@ -2305,7 +2267,7 @@
       </c>
       <c r="S13" s="21">
         <f t="shared" si="7"/>
-        <v>73.827922301309599</v>
+        <v>73.858245281309593</v>
       </c>
       <c r="T13" s="21">
         <f t="shared" si="8"/>
@@ -2313,7 +2275,7 @@
       </c>
       <c r="U13" s="21">
         <f t="shared" si="9"/>
-        <v>73.827922301309599</v>
+        <v>73.858245281309593</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.35">
@@ -2344,7 +2306,7 @@
       <c r="I14" s="42">
         <v>4.9630000000000001</v>
       </c>
-      <c r="J14" s="99">
+      <c r="J14" s="97">
         <v>76.745999999999995</v>
       </c>
       <c r="K14" s="20">
@@ -2380,7 +2342,7 @@
       </c>
       <c r="S14" s="21">
         <f t="shared" si="7"/>
-        <v>1285.2729059999988</v>
+        <v>1285.5066632999988</v>
       </c>
       <c r="T14" s="21">
         <f t="shared" si="8"/>
@@ -2388,7 +2350,7 @@
       </c>
       <c r="U14" s="21">
         <f t="shared" si="9"/>
-        <v>1285.2729059999988</v>
+        <v>1285.5066632999988</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.35">
@@ -2419,7 +2381,7 @@
       <c r="I15" s="42">
         <v>2.0644</v>
       </c>
-      <c r="J15" s="99">
+      <c r="J15" s="97">
         <v>0.53749999999999998</v>
       </c>
       <c r="K15" s="20">
@@ -2455,7 +2417,7 @@
       </c>
       <c r="S15" s="21">
         <f t="shared" si="7"/>
-        <v>-49.422247199994786</v>
+        <v>-49.325013959994749</v>
       </c>
       <c r="T15" s="21">
         <f t="shared" si="8"/>
@@ -2463,54 +2425,54 @@
       </c>
       <c r="U15" s="21">
         <f t="shared" si="9"/>
-        <v>-49.422247199994786</v>
+        <v>-49.325013959994749</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A16" s="106" t="s">
+      <c r="A16" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="101"/>
-      <c r="C16" s="101"/>
-      <c r="D16" s="103"/>
-      <c r="E16" s="101"/>
-      <c r="F16" s="101"/>
-      <c r="G16" s="101">
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="102"/>
+      <c r="F16" s="102"/>
+      <c r="G16" s="102">
         <f>'28-Euro Fund'!E10</f>
-        <v>460.46199999999999</v>
-      </c>
-      <c r="H16" s="101"/>
-      <c r="I16" s="101">
+        <v>460.50909999999999</v>
+      </c>
+      <c r="H16" s="102"/>
+      <c r="I16" s="102">
         <f>'28-Euro Fund'!D10</f>
         <v>156.44199999999998</v>
       </c>
-      <c r="J16" s="101"/>
-      <c r="K16" s="104"/>
-      <c r="L16" s="104"/>
-      <c r="M16" s="101"/>
-      <c r="N16" s="103"/>
-      <c r="O16" s="103"/>
-      <c r="P16" s="103"/>
-      <c r="Q16" s="103"/>
-      <c r="R16" s="103"/>
-      <c r="S16" s="103">
+      <c r="J16" s="102"/>
+      <c r="K16" s="100"/>
+      <c r="L16" s="100"/>
+      <c r="M16" s="102"/>
+      <c r="N16" s="99"/>
+      <c r="O16" s="99"/>
+      <c r="P16" s="99"/>
+      <c r="Q16" s="99"/>
+      <c r="R16" s="99"/>
+      <c r="S16" s="99">
         <f>SUM(S2:S15)</f>
-        <v>45659.294382907567</v>
-      </c>
-      <c r="T16" s="103"/>
-      <c r="U16" s="103"/>
-    </row>
-    <row r="17" spans="5:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>45666.662801107574</v>
+      </c>
+      <c r="T16" s="99"/>
+      <c r="U16" s="99"/>
+    </row>
+    <row r="17" spans="5:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="R17" s="13"/>
     </row>
-    <row r="18" spans="5:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E18" s="28" t="s">
         <v>31</v>
       </c>
       <c r="F18" s="29"/>
       <c r="G18" s="30"/>
     </row>
-    <row r="19" spans="5:18" x14ac:dyDescent="0.35">
+    <row r="19" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E19" s="41" t="s">
         <v>28</v>
       </c>
@@ -2520,8 +2482,11 @@
       <c r="G19" s="40" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="20" spans="5:18" x14ac:dyDescent="0.35">
+      <c r="R19" s="13"/>
+      <c r="S19" s="13"/>
+      <c r="T19" s="13"/>
+    </row>
+    <row r="20" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E20" s="33">
         <v>36871</v>
       </c>
@@ -2531,8 +2496,11 @@
       <c r="G20" s="34">
         <v>3087.53</v>
       </c>
-    </row>
-    <row r="21" spans="5:18" x14ac:dyDescent="0.35">
+      <c r="R20" s="13"/>
+      <c r="S20" s="13"/>
+      <c r="T20" s="13"/>
+    </row>
+    <row r="21" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E21" s="33">
         <v>36889</v>
       </c>
@@ -2542,8 +2510,11 @@
       <c r="G21" s="34">
         <v>3005.06</v>
       </c>
-    </row>
-    <row r="22" spans="5:18" x14ac:dyDescent="0.35">
+      <c r="R21" s="13"/>
+      <c r="S21" s="13"/>
+      <c r="T21" s="13"/>
+    </row>
+    <row r="22" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E22" s="33">
         <v>36913</v>
       </c>
@@ -2553,8 +2524,11 @@
       <c r="G22" s="34">
         <v>601.01</v>
       </c>
-    </row>
-    <row r="23" spans="5:18" x14ac:dyDescent="0.35">
+      <c r="R22" s="13"/>
+      <c r="S22" s="13"/>
+      <c r="T22" s="13"/>
+    </row>
+    <row r="23" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E23" s="33">
         <v>41169</v>
       </c>
@@ -2564,8 +2538,11 @@
       <c r="G23" s="34">
         <v>0.23</v>
       </c>
-    </row>
-    <row r="24" spans="5:18" x14ac:dyDescent="0.35">
+      <c r="R23" s="26"/>
+      <c r="S23" s="26"/>
+      <c r="T23" s="13"/>
+    </row>
+    <row r="24" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E24" s="31" t="s">
         <v>32</v>
       </c>
@@ -2577,8 +2554,10 @@
         <f>SUM(G20:G23)</f>
         <v>6693.83</v>
       </c>
-    </row>
-    <row r="25" spans="5:18" x14ac:dyDescent="0.35">
+      <c r="S24" s="26"/>
+      <c r="T24" s="13"/>
+    </row>
+    <row r="25" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E25" s="41" t="s">
         <v>30</v>
       </c>
@@ -2589,7 +2568,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="5:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="5:20" x14ac:dyDescent="0.35">
       <c r="E26" s="33">
         <v>45495</v>
       </c>
@@ -2600,7 +2579,7 @@
         <v>8530.48</v>
       </c>
     </row>
-    <row r="27" spans="5:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="5:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E27" s="36"/>
       <c r="F27" s="37" t="s">
         <v>9</v>
@@ -2610,7 +2589,7 @@
         <v>1836.6499999999996</v>
       </c>
     </row>
-    <row r="28" spans="5:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="5:20" x14ac:dyDescent="0.35">
       <c r="J28" s="27"/>
       <c r="K28" s="27"/>
     </row>
@@ -2664,14 +2643,14 @@
         <v>3</v>
       </c>
       <c r="F1" s="46" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G1" s="46"/>
       <c r="H1" s="46" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I1" s="46" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="J1" s="46"/>
       <c r="K1" s="46"/>
@@ -2687,7 +2666,7 @@
       <c r="C2" s="3">
         <v>45495</v>
       </c>
-      <c r="D2" s="71">
+      <c r="D2" s="70">
         <v>20.32</v>
       </c>
       <c r="E2" s="5">
@@ -2702,12 +2681,12 @@
       </c>
       <c r="I2" s="13">
         <f>(E3-E2)*D3</f>
-        <v>-55.12409600000003</v>
+        <v>-35.724592000000122</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B3" s="49" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C3" s="45"/>
       <c r="D3" s="32">
@@ -2715,15 +2694,15 @@
         <v>20.32</v>
       </c>
       <c r="E3" s="9">
-        <v>45.307400000000001</v>
+        <v>46.262099999999997</v>
       </c>
       <c r="F3" s="9">
         <f>D3*E3</f>
-        <v>920.64636800000005</v>
+        <v>940.04587199999992</v>
       </c>
       <c r="I3" s="26">
         <f>SUM(I2)</f>
-        <v>-55.12409600000003</v>
+        <v>-35.724592000000122</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -2796,11 +2775,11 @@
       <c r="I1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="91" t="s">
+      <c r="J1" s="89" t="s">
         <v>13</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>8</v>
@@ -2824,10 +2803,10 @@
         <v>19</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
@@ -2849,7 +2828,7 @@
       <c r="F2" s="19">
         <v>41166.000694444447</v>
       </c>
-      <c r="G2" s="88">
+      <c r="G2" s="86">
         <v>48.020240000000001</v>
       </c>
       <c r="H2" s="21">
@@ -2858,7 +2837,7 @@
       <c r="I2" s="54">
         <v>20.32</v>
       </c>
-      <c r="J2" s="92">
+      <c r="J2" s="90">
         <v>18.116299999999999</v>
       </c>
       <c r="K2" s="54">
@@ -2891,54 +2870,57 @@
         <v>0</v>
       </c>
       <c r="S2" s="21">
-        <f>N2*G$3-Q2</f>
-        <v>589.84273002514192</v>
+        <f>Q3-Q2</f>
+        <v>609.24223402514167</v>
       </c>
       <c r="T2" s="21">
         <f>R2+S2</f>
-        <v>589.84273002514192</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" s="12" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="101"/>
-      <c r="B3" s="101"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="102" t="s">
-        <v>44</v>
-      </c>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="103">
+        <v>609.24223402514167</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A3" s="101" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="99">
         <f>'1043-Global Tech US'!E3</f>
-        <v>45.307400000000001</v>
-      </c>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="101"/>
-      <c r="L3" s="101"/>
-      <c r="M3" s="101"/>
-      <c r="N3" s="104">
+        <v>46.262099999999997</v>
+      </c>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98">
+        <f>'1043-Global Tech US'!D3</f>
+        <v>20.32</v>
+      </c>
+      <c r="J3" s="98"/>
+      <c r="K3" s="100"/>
+      <c r="L3" s="100"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="100">
         <f>SUM(N2:N2)</f>
         <v>20.32</v>
       </c>
-      <c r="O3" s="104"/>
-      <c r="P3" s="101"/>
-      <c r="Q3" s="103">
-        <f>SUM(Q2:Q2)</f>
-        <v>330.80363797485819</v>
-      </c>
-      <c r="R3" s="103">
+      <c r="O3" s="99"/>
+      <c r="P3" s="99"/>
+      <c r="Q3" s="99">
+        <f>N3*G3</f>
+        <v>940.04587199999992</v>
+      </c>
+      <c r="R3" s="99">
         <f>SUM(R2:R2)</f>
         <v>0</v>
       </c>
-      <c r="S3" s="103">
+      <c r="S3" s="99">
         <f>SUM(S2:S2)</f>
-        <v>589.84273002514192</v>
-      </c>
-      <c r="T3" s="103">
+        <v>609.24223402514167</v>
+      </c>
+      <c r="T3" s="99">
         <f>SUM(T2:T2)</f>
-        <v>589.84273002514192</v>
+        <v>609.24223402514167</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="12" customFormat="1" x14ac:dyDescent="0.35">
@@ -2972,7 +2954,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.08984375" customWidth="1"/>
@@ -3000,29 +2982,29 @@
         <v>3</v>
       </c>
       <c r="F1" s="46" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G1" s="46"/>
       <c r="H1" s="46" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I1" s="46" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J1" s="46" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="L1" s="46" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="M1" s="46" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="N1" s="46" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="O1" s="46"/>
       <c r="P1" s="46"/>
@@ -3070,11 +3052,11 @@
       </c>
       <c r="M2" s="13">
         <f>(E12-E2)*J2</f>
-        <v>4103.7644000000046</v>
+        <v>4241.7405000000044</v>
       </c>
       <c r="N2" s="27">
         <f>L2+M2</f>
-        <v>32126.966400000001</v>
+        <v>32264.942500000001</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
@@ -3082,7 +3064,7 @@
         <v>198</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C3" s="3">
         <v>44470</v>
@@ -3112,7 +3094,7 @@
         <v>200</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C4" s="3">
         <v>44473</v>
@@ -3142,7 +3124,7 @@
         <v>216</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C5" s="3">
         <v>44720</v>
@@ -3170,7 +3152,7 @@
         <v>1227</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C6" s="3">
         <v>44831</v>
@@ -3198,7 +3180,7 @@
         <v>1247</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C7" s="3">
         <v>45028</v>
@@ -3287,11 +3269,11 @@
       </c>
       <c r="M9" s="13">
         <f>(E$12-E9)*J9</f>
-        <v>578.28009666000139</v>
+        <v>847.53599666000082</v>
       </c>
       <c r="N9" s="27">
         <f>L9+M9</f>
-        <v>578.28009666000139</v>
+        <v>847.53599666000082</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.35">
@@ -3332,11 +3314,11 @@
       </c>
       <c r="M10" s="13">
         <f>(E$12-E10)*J10</f>
-        <v>-708.01468725399991</v>
+        <v>-403.73198725400056</v>
       </c>
       <c r="N10" s="27">
         <f>L10+M10</f>
-        <v>-708.01468725399991</v>
+        <v>-403.73198725400056</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
@@ -3344,7 +3326,7 @@
         <v>1279</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C11" s="3">
         <v>45495</v>
@@ -3369,7 +3351,7 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B12" s="49" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C12" s="45"/>
       <c r="D12" s="32">
@@ -3377,11 +3359,11 @@
         <v>704.47</v>
       </c>
       <c r="E12" s="9">
-        <v>47.09</v>
+        <v>48.1</v>
       </c>
       <c r="F12" s="9">
         <f>D12*E12</f>
-        <v>33173.492300000005</v>
+        <v>33885.007000000005</v>
       </c>
       <c r="J12" s="32">
         <f>SUM(J2:J11)</f>
@@ -3393,7 +3375,7 @@
     </row>
     <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="J13" s="8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="K13" s="26">
         <f>SUM(K2:K12)</f>
@@ -3405,17 +3387,17 @@
       </c>
       <c r="M13" s="26">
         <f>SUM(M2:M12)</f>
-        <v>3974.0298094060063</v>
+        <v>4685.5445094060051</v>
       </c>
       <c r="N13" s="50">
         <f>SUM(N2:N12)</f>
-        <v>31997.231809406003</v>
+        <v>32708.746509405999</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D14" s="51"/>
       <c r="E14" s="52" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F14" s="53">
         <f>D8*(E8-E2)</f>
@@ -3426,309 +3408,39 @@
     <row r="15" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D15" s="51"/>
       <c r="E15" s="52" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F15" s="53">
         <f>D11*(E11-E2)</f>
         <v>634.99999999999989</v>
       </c>
       <c r="H15" s="12"/>
-      <c r="I15">
-        <v>173</v>
-      </c>
-      <c r="J15" s="10">
-        <f>J2*E2</f>
-        <v>2329.2005000000022</v>
-      </c>
+      <c r="J15" s="10"/>
       <c r="K15" s="10"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="F16" s="10"/>
-      <c r="I16">
-        <v>1273</v>
-      </c>
-      <c r="J16" s="10">
-        <f>J9*E9</f>
-        <v>11975.443003339999</v>
-      </c>
+      <c r="J16" s="10"/>
       <c r="K16" s="10"/>
-      <c r="L16" s="66">
-        <v>238.36680000000001</v>
-      </c>
-      <c r="M16" s="66">
-        <v>28.223199999999999</v>
-      </c>
-      <c r="N16" s="67">
-        <f>+L16+M16</f>
-        <v>266.59000000000003</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="I17">
-        <v>1275</v>
-      </c>
-      <c r="J17" s="10">
-        <f>J10*E10</f>
-        <v>14894.818987254001</v>
-      </c>
+      <c r="L16" s="66"/>
+      <c r="M16" s="66"/>
+      <c r="N16" s="67"/>
+    </row>
+    <row r="17" spans="10:15" x14ac:dyDescent="0.35">
+      <c r="J17" s="10"/>
       <c r="K17" s="10"/>
-      <c r="L17" s="66">
-        <v>97.849199999999996</v>
-      </c>
-      <c r="M17" s="66">
-        <v>20.558299999999999</v>
-      </c>
-      <c r="N17" s="66">
-        <v>182.86250000000001</v>
-      </c>
-      <c r="O17" s="67">
-        <f>SUM(L17:N17)</f>
-        <v>301.27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="J18" s="68">
-        <f>SUM(J15:J17)</f>
-        <v>29199.462490594</v>
-      </c>
+      <c r="L17" s="66"/>
+      <c r="M17" s="66"/>
+      <c r="N17" s="66"/>
+      <c r="O17" s="67"/>
+    </row>
+    <row r="18" spans="10:15" x14ac:dyDescent="0.35">
+      <c r="J18" s="68"/>
       <c r="K18" s="68"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="10:15" x14ac:dyDescent="0.35">
       <c r="J19" s="10"/>
       <c r="K19" s="10"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A20" s="72" t="s">
-        <v>64</v>
-      </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A21" s="1">
-        <v>1263</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C21" s="3">
-        <v>45209</v>
-      </c>
-      <c r="D21" s="1">
-        <v>116.8907</v>
-      </c>
-      <c r="E21" s="5">
-        <v>85.55</v>
-      </c>
-      <c r="F21" s="5">
-        <v>10000</v>
-      </c>
-      <c r="J21" s="12">
-        <f>D21</f>
-        <v>116.8907</v>
-      </c>
-      <c r="K21" s="10"/>
-      <c r="M21" s="10">
-        <f>(E22-E21)*J21</f>
-        <v>439.50903200000056</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E22" s="70">
-        <v>89.31</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A23" s="45" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A24" s="1">
-        <v>1280</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C24" s="3">
-        <v>45495</v>
-      </c>
-      <c r="D24" s="1">
-        <v>20.32</v>
-      </c>
-      <c r="E24" s="5">
-        <v>48.020200000000003</v>
-      </c>
-      <c r="F24" s="5">
-        <v>975.77</v>
-      </c>
-      <c r="J24" s="12">
-        <f>D24</f>
-        <v>20.32</v>
-      </c>
-      <c r="K24" s="10"/>
-      <c r="M24" s="10">
-        <f>(E25-E24)*J24</f>
-        <v>-49.601120000000051</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E25" s="9">
-        <v>45.5792</v>
-      </c>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A26" s="45" t="s">
-        <v>66</v>
-      </c>
-      <c r="I26" s="45" t="s">
-        <v>69</v>
-      </c>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="N26" s="45" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A27" s="1">
-        <v>1286</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C27" s="3">
-        <v>45539</v>
-      </c>
-      <c r="D27" s="1">
-        <v>50</v>
-      </c>
-      <c r="E27" s="5">
-        <v>19.97</v>
-      </c>
-      <c r="F27" s="5">
-        <v>998.5</v>
-      </c>
-      <c r="G27" s="5">
-        <v>1005.78</v>
-      </c>
-      <c r="H27" s="1"/>
-      <c r="I27" s="5">
-        <v>7.28</v>
-      </c>
-      <c r="J27" s="12">
-        <f>D27</f>
-        <v>50</v>
-      </c>
-      <c r="K27" s="10"/>
-      <c r="M27" s="10">
-        <f>(E28-E27)*J27</f>
-        <v>27.000000000000135</v>
-      </c>
-      <c r="N27" s="10">
-        <f>M27-I27</f>
-        <v>19.720000000000134</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E28" s="9">
-        <v>20.51</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A29" s="45" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A30" s="1">
-        <v>1288</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C30" s="3">
-        <v>45545</v>
-      </c>
-      <c r="D30" s="73">
-        <v>1000</v>
-      </c>
-      <c r="E30" s="5">
-        <v>19.899999999999999</v>
-      </c>
-      <c r="F30" s="5">
-        <v>19900</v>
-      </c>
-      <c r="G30" s="5">
-        <v>19901</v>
-      </c>
-      <c r="H30" s="1"/>
-      <c r="I30" s="5">
-        <v>1</v>
-      </c>
-      <c r="J30" s="12">
-        <f>D30</f>
-        <v>1000</v>
-      </c>
-      <c r="K30" s="10"/>
-      <c r="M30" s="10">
-        <f>(E31-E30)*J30</f>
-        <v>614.0000000000008</v>
-      </c>
-      <c r="N30" s="10">
-        <f>M30-I30</f>
-        <v>613.0000000000008</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E31" s="9">
-        <v>20.513999999999999</v>
-      </c>
-    </row>
-    <row r="33" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E33" t="s">
-        <v>1</v>
-      </c>
-      <c r="F33">
-        <v>11025.76</v>
-      </c>
-    </row>
-    <row r="34" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E34" t="s">
-        <v>62</v>
-      </c>
-      <c r="F34">
-        <v>9979.52</v>
-      </c>
-    </row>
-    <row r="35" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="F35">
-        <f>+F33-F34</f>
-        <v>1046.2399999999998</v>
-      </c>
-    </row>
-    <row r="37" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E37">
-        <v>469.02</v>
-      </c>
-    </row>
-    <row r="38" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E38">
-        <v>482.6</v>
-      </c>
-    </row>
-    <row r="39" spans="5:6" x14ac:dyDescent="0.35">
-      <c r="E39">
-        <f>+E37-E38</f>
-        <v>-13.580000000000041</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3741,7 +3453,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:AD34"/>
+  <dimension ref="A1:AD33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.7265625" customWidth="1"/>
@@ -3792,11 +3504,11 @@
       <c r="I1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="91" t="s">
+      <c r="J1" s="89" t="s">
         <v>13</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>8</v>
@@ -3820,10 +3532,10 @@
         <v>19</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
@@ -3845,7 +3557,7 @@
       <c r="F2" s="19">
         <v>36841</v>
       </c>
-      <c r="G2" s="88">
+      <c r="G2" s="86">
         <v>17.05</v>
       </c>
       <c r="H2" s="21">
@@ -3854,7 +3566,7 @@
       <c r="I2" s="54">
         <v>544.952</v>
       </c>
-      <c r="J2" s="92">
+      <c r="J2" s="90">
         <v>679.64009999999996</v>
       </c>
       <c r="K2" s="54">
@@ -3900,14 +3612,14 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="89">
+        <v>46</v>
+      </c>
+      <c r="B3" s="87">
         <v>198</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
-      <c r="E3" s="90">
+      <c r="E3" s="88">
         <v>44470</v>
       </c>
       <c r="F3" s="22"/>
@@ -3918,7 +3630,7 @@
       <c r="I3" s="56">
         <v>287.02999999999997</v>
       </c>
-      <c r="J3" s="93"/>
+      <c r="J3" s="91"/>
       <c r="K3" s="56">
         <f>I3</f>
         <v>287.02999999999997</v>
@@ -3938,14 +3650,14 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="89">
+        <v>46</v>
+      </c>
+      <c r="B4" s="87">
         <v>200</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="22"/>
-      <c r="E4" s="90">
+      <c r="E4" s="88">
         <v>44473</v>
       </c>
       <c r="F4" s="22"/>
@@ -3956,7 +3668,7 @@
       <c r="I4" s="56">
         <v>287.02999999999997</v>
       </c>
-      <c r="J4" s="93"/>
+      <c r="J4" s="91"/>
       <c r="K4" s="56">
         <f>I2-K3</f>
         <v>257.92200000000003</v>
@@ -3993,7 +3705,7 @@
       <c r="F5" s="19">
         <v>41166</v>
       </c>
-      <c r="G5" s="88">
+      <c r="G5" s="86">
         <v>17.05</v>
       </c>
       <c r="H5" s="21">
@@ -4002,7 +3714,7 @@
       <c r="I5" s="18">
         <v>1065.5911000000001</v>
       </c>
-      <c r="J5" s="92">
+      <c r="J5" s="90">
         <v>547.64509999999996</v>
       </c>
       <c r="K5" s="20">
@@ -4048,14 +3760,14 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="89">
+        <v>46</v>
+      </c>
+      <c r="B6" s="87">
         <v>200</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
-      <c r="E6" s="90">
+      <c r="E6" s="88">
         <v>44473</v>
       </c>
       <c r="F6" s="22"/>
@@ -4066,7 +3778,7 @@
       <c r="I6" s="56">
         <v>287.02999999999997</v>
       </c>
-      <c r="J6" s="93"/>
+      <c r="J6" s="91"/>
       <c r="K6" s="56">
         <f>I6-K4</f>
         <v>29.107999999999947</v>
@@ -4086,14 +3798,14 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="89">
+        <v>46</v>
+      </c>
+      <c r="B7" s="87">
         <v>216</v>
       </c>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
-      <c r="E7" s="90">
+      <c r="E7" s="88">
         <v>44720</v>
       </c>
       <c r="F7" s="22"/>
@@ -4104,7 +3816,7 @@
       <c r="I7" s="56">
         <v>296.82</v>
       </c>
-      <c r="J7" s="93"/>
+      <c r="J7" s="91"/>
       <c r="K7" s="56">
         <f>I7</f>
         <v>296.82</v>
@@ -4124,14 +3836,14 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="89">
+        <v>46</v>
+      </c>
+      <c r="B8" s="87">
         <v>1227</v>
       </c>
       <c r="C8" s="22"/>
       <c r="D8" s="22"/>
-      <c r="E8" s="90">
+      <c r="E8" s="88">
         <v>44831</v>
       </c>
       <c r="F8" s="22"/>
@@ -4142,7 +3854,7 @@
       <c r="I8" s="56">
         <v>308.74</v>
       </c>
-      <c r="J8" s="93"/>
+      <c r="J8" s="91"/>
       <c r="K8" s="56">
         <f>I8</f>
         <v>308.74</v>
@@ -4162,14 +3874,14 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" s="89">
+        <v>46</v>
+      </c>
+      <c r="B9" s="87">
         <v>1247</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
-      <c r="E9" s="90">
+      <c r="E9" s="88">
         <v>45028</v>
       </c>
       <c r="F9" s="22"/>
@@ -4180,7 +3892,7 @@
       <c r="I9" s="56">
         <v>172.46</v>
       </c>
-      <c r="J9" s="93"/>
+      <c r="J9" s="91"/>
       <c r="K9" s="56">
         <f>I9</f>
         <v>172.46</v>
@@ -4202,12 +3914,12 @@
       <c r="A10" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="89">
+      <c r="B10" s="87">
         <v>1251</v>
       </c>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
-      <c r="E10" s="90">
+      <c r="E10" s="88">
         <v>45054</v>
       </c>
       <c r="F10" s="22"/>
@@ -4218,7 +3930,7 @@
       <c r="I10" s="56">
         <v>270</v>
       </c>
-      <c r="J10" s="93"/>
+      <c r="J10" s="91"/>
       <c r="K10" s="56"/>
       <c r="L10" s="56">
         <f>I5-K5</f>
@@ -4255,7 +3967,7 @@
       <c r="F11" s="19">
         <v>41377</v>
       </c>
-      <c r="G11" s="88">
+      <c r="G11" s="86">
         <v>17.05</v>
       </c>
       <c r="H11" s="21">
@@ -4264,7 +3976,7 @@
       <c r="I11" s="54">
         <v>168.14699999999999</v>
       </c>
-      <c r="J11" s="92">
+      <c r="J11" s="90">
         <v>86.4482</v>
       </c>
       <c r="K11" s="18"/>
@@ -4298,23 +4010,23 @@
       </c>
       <c r="S11" s="21">
         <f>N11*G$19-Q11</f>
-        <v>5781.341933011352</v>
+        <v>5939.5181340113504</v>
       </c>
       <c r="T11" s="21">
         <f>R11+S11</f>
-        <v>6059.5601765634983</v>
+        <v>6217.7363775634967</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="89">
+      <c r="B12" s="87">
         <v>1251</v>
       </c>
       <c r="C12" s="22"/>
       <c r="D12" s="22"/>
-      <c r="E12" s="90">
+      <c r="E12" s="88">
         <v>45054</v>
       </c>
       <c r="F12" s="22"/>
@@ -4325,7 +4037,7 @@
       <c r="I12" s="56">
         <v>270</v>
       </c>
-      <c r="J12" s="94"/>
+      <c r="J12" s="92"/>
       <c r="K12" s="24"/>
       <c r="L12" s="56">
         <f>I12-L10</f>
@@ -4362,7 +4074,7 @@
       <c r="F13" s="19">
         <v>41166</v>
       </c>
-      <c r="G13" s="88">
+      <c r="G13" s="86">
         <v>49.440100000000001</v>
       </c>
       <c r="H13" s="21">
@@ -4371,7 +4083,7 @@
       <c r="I13" s="54">
         <v>97.849000000000004</v>
       </c>
-      <c r="J13" s="92">
+      <c r="J13" s="90">
         <v>88.633300000000006</v>
       </c>
       <c r="K13" s="54">
@@ -4408,23 +4120,23 @@
       </c>
       <c r="S13" s="21">
         <f>N13*G$19-Q13</f>
-        <v>2378.2697666549875</v>
+        <v>2456.8972566549874</v>
       </c>
       <c r="T13" s="21">
         <f>R13+S13</f>
-        <v>2378.2697666549875</v>
+        <v>2456.8972566549874</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="89">
+        <v>46</v>
+      </c>
+      <c r="B14" s="87">
         <v>1279</v>
       </c>
       <c r="C14" s="22"/>
       <c r="D14" s="22"/>
-      <c r="E14" s="90">
+      <c r="E14" s="88">
         <v>45495</v>
       </c>
       <c r="F14" s="22"/>
@@ -4435,7 +4147,7 @@
       <c r="I14" s="56">
         <v>20</v>
       </c>
-      <c r="J14" s="93"/>
+      <c r="J14" s="91"/>
       <c r="K14" s="56">
         <f>I14</f>
         <v>20</v>
@@ -4481,10 +4193,10 @@
       <c r="I15" s="54">
         <v>238.36699999999999</v>
       </c>
-      <c r="J15" s="95">
+      <c r="J15" s="93">
         <v>264.64670000000001</v>
       </c>
-      <c r="K15" s="97"/>
+      <c r="K15" s="95"/>
       <c r="L15" s="54">
         <v>0</v>
       </c>
@@ -4513,11 +4225,11 @@
       </c>
       <c r="S15" s="21">
         <f>N15*G$19-Q15</f>
-        <v>5987.3442795569526</v>
+        <v>6228.0949495569521</v>
       </c>
       <c r="T15" s="21">
         <f t="shared" ref="T15:T18" si="3">R15+S15</f>
-        <v>5987.3442795569526</v>
+        <v>6228.0949495569521</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.35">
@@ -4548,7 +4260,7 @@
       <c r="I16" s="54">
         <v>28.222999999999999</v>
       </c>
-      <c r="J16" s="96">
+      <c r="J16" s="94">
         <v>45.477400000000003</v>
       </c>
       <c r="K16" s="54"/>
@@ -4580,11 +4292,11 @@
       </c>
       <c r="S16" s="21">
         <f>N16*G$19-Q16</f>
-        <v>551.6639672342834</v>
+        <v>580.16919723428339</v>
       </c>
       <c r="T16" s="21">
         <f t="shared" si="3"/>
-        <v>551.6639672342834</v>
+        <v>580.16919723428339</v>
       </c>
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.35">
@@ -4598,7 +4310,7 @@
         <v>1253</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E17" s="19">
         <v>45478</v>
@@ -4615,10 +4327,10 @@
       <c r="I17" s="54">
         <v>20.558</v>
       </c>
-      <c r="J17" s="95">
+      <c r="J17" s="93">
         <v>8.4095999999999993</v>
       </c>
-      <c r="K17" s="97"/>
+      <c r="K17" s="95"/>
       <c r="L17" s="54">
         <v>0</v>
       </c>
@@ -4647,11 +4359,11 @@
       </c>
       <c r="S17" s="21">
         <f>N17*G$19-Q17</f>
-        <v>-31.949909139199917</v>
+        <v>-11.186329139199984</v>
       </c>
       <c r="T17" s="21">
         <f t="shared" si="3"/>
-        <v>-31.949909139199917</v>
+        <v>-11.186329139199984</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.35">
@@ -4665,7 +4377,7 @@
         <v>1254</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E18" s="19">
         <v>45478</v>
@@ -4682,10 +4394,10 @@
       <c r="I18" s="54">
         <v>182.863</v>
       </c>
-      <c r="J18" s="95">
+      <c r="J18" s="93">
         <v>74.801699999999997</v>
       </c>
-      <c r="K18" s="97"/>
+      <c r="K18" s="95"/>
       <c r="L18" s="54">
         <v>0</v>
       </c>
@@ -4714,216 +4426,221 @@
       </c>
       <c r="S18" s="21">
         <f>N18*G$19-Q18</f>
-        <v>-388.97531502918901</v>
+        <v>-204.28368502918966</v>
       </c>
       <c r="T18" s="21">
         <f t="shared" si="3"/>
-        <v>-388.97531502918901</v>
-      </c>
-    </row>
-    <row r="19" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="101"/>
-      <c r="B19" s="101"/>
-      <c r="C19" s="101"/>
-      <c r="D19" s="102" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="101"/>
-      <c r="F19" s="101"/>
-      <c r="G19" s="103">
+        <v>-204.28368502918966</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="A19" s="101" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="98"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="99"/>
+      <c r="E19" s="98"/>
+      <c r="F19" s="98"/>
+      <c r="G19" s="99">
         <f>'27-Global Tech EU'!E12</f>
-        <v>47.09</v>
-      </c>
-      <c r="H19" s="101"/>
-      <c r="I19" s="101"/>
-      <c r="J19" s="101"/>
-      <c r="K19" s="101"/>
-      <c r="L19" s="101"/>
-      <c r="M19" s="101"/>
-      <c r="N19" s="104">
+        <v>48.1</v>
+      </c>
+      <c r="H19" s="98"/>
+      <c r="I19" s="98"/>
+      <c r="J19" s="98"/>
+      <c r="K19" s="100"/>
+      <c r="L19" s="100"/>
+      <c r="M19" s="98"/>
+      <c r="N19" s="100">
         <f>SUM(N2:N18)</f>
         <v>704.47010000000023</v>
       </c>
-      <c r="O19" s="104"/>
-      <c r="P19" s="101"/>
-      <c r="Q19" s="103">
+      <c r="O19" s="99"/>
+      <c r="P19" s="99"/>
+      <c r="Q19" s="99">
         <f>SUM(Q2:Q18)</f>
         <v>18895.802286710823</v>
       </c>
-      <c r="R19" s="103">
+      <c r="R19" s="99">
         <f>SUM(R2:R18)</f>
         <v>6715.3807197918886</v>
       </c>
-      <c r="S19" s="103">
+      <c r="S19" s="99">
         <f>SUM(S2:S18)</f>
-        <v>14277.694722289185</v>
-      </c>
-      <c r="T19" s="103">
+        <v>14989.209523289182</v>
+      </c>
+      <c r="T19" s="99">
         <f>SUM(T2:T18)</f>
-        <v>20993.075442081077</v>
-      </c>
-    </row>
-    <row r="20" spans="1:30" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C20" s="32"/>
-      <c r="N20" s="57"/>
-      <c r="O20" s="58"/>
-      <c r="Q20" s="26"/>
-      <c r="S20" s="26">
-        <v>13883.187</v>
-      </c>
-    </row>
-    <row r="21" spans="1:30" s="12" customFormat="1" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C21" s="84"/>
-      <c r="D21" s="86" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="85"/>
+        <v>21704.590243081075</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30" s="12" customFormat="1" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="AA20" s="57"/>
+      <c r="AD20" s="57"/>
+    </row>
+    <row r="21" spans="1:30" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O21" s="59" t="s">
+        <v>49</v>
+      </c>
+      <c r="P21" s="60"/>
+      <c r="S21" s="103" t="s">
+        <v>65</v>
+      </c>
+      <c r="T21" s="104">
+        <f>+T15+T16</f>
+        <v>6808.2641467912354</v>
+      </c>
       <c r="AA21" s="57"/>
       <c r="AD21" s="57"/>
     </row>
-    <row r="22" spans="1:30" s="12" customFormat="1" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C22" s="87" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="79" t="s">
-        <v>55</v>
-      </c>
-      <c r="E22" s="78" t="s">
-        <v>56</v>
-      </c>
-      <c r="O22" s="59" t="s">
-        <v>54</v>
-      </c>
-      <c r="P22" s="60"/>
+    <row r="22" spans="1:30" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O22" s="61" t="s">
+        <v>52</v>
+      </c>
+      <c r="P22" s="62">
+        <f>SUM(R2:R11)</f>
+        <v>6715.3807197918886</v>
+      </c>
+      <c r="S22" s="105" t="s">
+        <v>66</v>
+      </c>
+      <c r="T22" s="106">
+        <f>+T18+T17+T13</f>
+        <v>2241.4272424865976</v>
+      </c>
       <c r="AA22" s="57"/>
       <c r="AD22" s="57"/>
     </row>
-    <row r="23" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C23" s="80">
-        <v>16</v>
-      </c>
-      <c r="D23" s="12">
-        <f>J5/I5*L10</f>
-        <v>132.83336379762375</v>
-      </c>
-      <c r="E23" s="76">
-        <f>D23*H5</f>
-        <v>2425.5372227602638</v>
-      </c>
+    <row r="23" spans="1:30" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="O23" s="61" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="P23" s="62">
-        <f>SUM(R2:R11)</f>
-        <v>6715.3807197918886</v>
+        <f>SUM(S2:S11)</f>
+        <v>5939.5181340113504</v>
       </c>
       <c r="AA23" s="57"/>
       <c r="AD23" s="57"/>
     </row>
-    <row r="24" spans="1:30" s="12" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C24" s="81">
-        <v>17</v>
-      </c>
-      <c r="D24" s="82">
-        <f>J11/I11*L12</f>
-        <v>5.9313828886628102</v>
-      </c>
-      <c r="E24" s="83">
-        <f>D24*H11</f>
-        <v>117.38205744784817</v>
-      </c>
-      <c r="O24" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="P24" s="62">
-        <f>SUM(S2:S11)</f>
-        <v>5781.341933011352</v>
-      </c>
-      <c r="AA24" s="57"/>
-      <c r="AD24" s="57"/>
+    <row r="24" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F24" s="12"/>
+      <c r="O24" s="63" t="s">
+        <v>32</v>
+      </c>
+      <c r="P24" s="64">
+        <f>SUM(P22:P23)</f>
+        <v>12654.898853803239</v>
+      </c>
+      <c r="Y24" s="12"/>
     </row>
     <row r="25" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C25" s="51"/>
-      <c r="D25" s="52" t="s">
-        <v>71</v>
-      </c>
-      <c r="E25" s="77">
-        <f>SUM(E23:E24)</f>
-        <v>2542.919280208112</v>
-      </c>
       <c r="F25" s="12"/>
-      <c r="O25" s="63" t="s">
-        <v>32</v>
-      </c>
-      <c r="P25" s="64">
-        <f>SUM(P23:P24)</f>
-        <v>12496.722652803241</v>
-      </c>
-      <c r="Y25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
     </row>
     <row r="26" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C26" s="74"/>
-      <c r="D26" s="75" t="s">
-        <v>72</v>
-      </c>
-      <c r="E26" s="76">
-        <f>'27-Global Tech EU'!F8</f>
-        <v>9258.2999999999993</v>
-      </c>
       <c r="F26" s="12"/>
       <c r="J26" s="12"/>
       <c r="K26" s="12"/>
       <c r="L26" s="12"/>
-    </row>
-    <row r="27" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C27" s="51"/>
-      <c r="D27" s="52" t="s">
-        <v>70</v>
-      </c>
-      <c r="E27" s="64">
-        <f>E26-E25</f>
-        <v>6715.3807197918868</v>
-      </c>
+      <c r="O26" s="82"/>
+      <c r="P26" s="84" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q26" s="83"/>
+    </row>
+    <row r="27" spans="1:30" ht="29" x14ac:dyDescent="0.35">
       <c r="F27" s="12"/>
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
       <c r="L27" s="12"/>
+      <c r="O27" s="85" t="s">
+        <v>5</v>
+      </c>
+      <c r="P27" s="77" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q27" s="76" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.35">
       <c r="F28" s="12"/>
       <c r="J28" s="12"/>
       <c r="K28" s="12"/>
       <c r="L28" s="12"/>
-    </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="O28" s="78">
+        <v>16</v>
+      </c>
+      <c r="P28" s="12">
+        <f>J5/I5*L10</f>
+        <v>132.83336379762375</v>
+      </c>
+      <c r="Q28" s="74">
+        <f>P28*H5</f>
+        <v>2425.5372227602638</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F29" s="12"/>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
       <c r="L29" s="12"/>
-    </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.35">
-      <c r="F30" s="12"/>
+      <c r="O29" s="79">
+        <v>17</v>
+      </c>
+      <c r="P29" s="80">
+        <f>J11/I11*L12</f>
+        <v>5.9313828886628102</v>
+      </c>
+      <c r="Q29" s="81">
+        <f>P29*H11</f>
+        <v>117.38205744784817</v>
+      </c>
+    </row>
+    <row r="30" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
       <c r="L30" s="12"/>
-    </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="O30" s="51"/>
+      <c r="P30" s="52" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q30" s="75">
+        <f>SUM(Q28:Q29)</f>
+        <v>2542.919280208112</v>
+      </c>
+    </row>
+    <row r="31" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
       <c r="L31" s="12"/>
-    </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.35">
+      <c r="O31" s="72"/>
+      <c r="P31" s="73" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q31" s="74">
+        <f>'27-Global Tech EU'!F8</f>
+        <v>9258.2999999999993</v>
+      </c>
+    </row>
+    <row r="32" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
-      <c r="L32" s="12"/>
+      <c r="O32" s="51"/>
+      <c r="P32" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q32" s="64">
+        <f>Q31-Q30</f>
+        <v>6715.3807197918868</v>
+      </c>
     </row>
     <row r="33" spans="10:11" x14ac:dyDescent="0.35">
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
-    </row>
-    <row r="34" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4944,7 +4661,7 @@
   <cols>
     <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" customWidth="1"/>
     <col min="7" max="7" width="2.6328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4959,7 +4676,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="46" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -4967,7 +4684,7 @@
         <v>1263</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C2" s="3">
         <v>45209</v>
@@ -4992,11 +4709,11 @@
         <v>116.8907</v>
       </c>
       <c r="E3" s="5">
-        <v>89.34</v>
+        <v>89.37</v>
       </c>
       <c r="F3" s="5">
         <f>D3*E3</f>
-        <v>10443.015138000001</v>
+        <v>10446.521859</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -5005,7 +4722,7 @@
       </c>
       <c r="F4" s="4">
         <f>F3-F2</f>
-        <v>443.01513800000066</v>
+        <v>446.5218590000004</v>
       </c>
     </row>
   </sheetData>
@@ -5019,7 +4736,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
@@ -5035,7 +4752,8 @@
     <col min="13" max="13" width="9.1796875" customWidth="1"/>
     <col min="14" max="14" width="8.54296875" customWidth="1"/>
     <col min="15" max="15" width="10.7265625" customWidth="1"/>
-    <col min="16" max="17" width="11.36328125" customWidth="1"/>
+    <col min="16" max="16" width="11.36328125" customWidth="1"/>
+    <col min="17" max="17" width="11.7265625" customWidth="1"/>
     <col min="18" max="18" width="10.453125" customWidth="1"/>
     <col min="19" max="19" width="9.81640625" customWidth="1"/>
     <col min="20" max="20" width="10.54296875" bestFit="1" customWidth="1"/>
@@ -5069,11 +4787,11 @@
       <c r="I1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="98" t="s">
+      <c r="J1" s="96" t="s">
         <v>13</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>8</v>
@@ -5097,15 +4815,15 @@
         <v>19</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B2" s="18">
         <v>1263</v>
@@ -5114,7 +4832,7 @@
         <v>1263</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="E2" s="19">
         <v>45209.585717592592</v>
@@ -5131,7 +4849,7 @@
       <c r="I2" s="18">
         <v>116.8907</v>
       </c>
-      <c r="J2" s="92">
+      <c r="J2" s="90">
         <v>116.8907</v>
       </c>
       <c r="K2" s="18"/>
@@ -5165,74 +4883,57 @@
       </c>
       <c r="S2" s="21">
         <f>Q3-Q2</f>
-        <v>443.0157530000015</v>
+        <v>446.52247400000124</v>
       </c>
       <c r="T2" s="21">
         <f>R2+S2</f>
-        <v>443.0157530000015</v>
+        <v>446.52247400000124</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="25">
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="99">
         <f>'1042-DWS Floating'!E3</f>
-        <v>89.34</v>
-      </c>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="105"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25">
-        <f>N2*G3</f>
-        <v>10443.015138000001</v>
-      </c>
-      <c r="R3" s="25"/>
-      <c r="S3" s="25"/>
-      <c r="T3" s="25"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="N5" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="O5" s="45" t="s">
-        <v>37</v>
+        <v>89.37</v>
+      </c>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="100"/>
+      <c r="L3" s="100"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="100">
+        <f>SUM(N2)</f>
+        <v>116.8907</v>
+      </c>
+      <c r="O3" s="99"/>
+      <c r="P3" s="99"/>
+      <c r="Q3" s="99">
+        <f>N3*G3</f>
+        <v>10446.521859</v>
+      </c>
+      <c r="R3" s="99">
+        <f>SUM(R2)</f>
+        <v>0</v>
+      </c>
+      <c r="S3" s="99">
+        <f t="shared" ref="S3:T3" si="0">SUM(S2)</f>
+        <v>446.52247400000124</v>
+      </c>
+      <c r="T3" s="99">
+        <f t="shared" si="0"/>
+        <v>446.52247400000124</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="N6">
-        <v>29</v>
-      </c>
-      <c r="O6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="N7">
-        <v>28</v>
-      </c>
-      <c r="O7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="L8" s="45"/>
-      <c r="O8" s="45" t="s">
-        <v>40</v>
-      </c>
+      <c r="M6" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>